<commit_message>
feat: implementar generación de archivo de anexo por separado en la acción de nómina de pago, mejorando la organización y manejo de archivos generados
</commit_message>
<xml_diff>
--- a/src/core/excel/templates/ANEXO NOMINA DE PAGO PERSONAL DIRECTIVO.xlsx
+++ b/src/core/excel/templates/ANEXO NOMINA DE PAGO PERSONAL DIRECTIVO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\OneDrive\Documentos\Codigo\san-miguel-porres-backend\src\core\excel\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A0FA9A79-D1B6-487E-BF1E-23BD812CE88B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A838FAB-D092-40B8-8E5A-627DC3D0F25A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
   <si>
     <t>ANEXO-NP1</t>
   </si>
@@ -131,9 +131,6 @@
   </si>
   <si>
     <t>RECONVERSIÓN DE HORAS A 40</t>
-  </si>
-  <si>
-    <t>.</t>
   </si>
   <si>
     <t>TIEMPO SERVICIO</t>
@@ -206,6 +203,18 @@
   </si>
   <si>
     <t>ANALISIS / julio 2023</t>
+  </si>
+  <si>
+    <t>PUNTAJE</t>
+  </si>
+  <si>
+    <t>CARGO</t>
+  </si>
+  <si>
+    <t>Nº HRAS SEMAN</t>
+  </si>
+  <si>
+    <t>CATEG. DOCENTE</t>
   </si>
 </sst>
 </file>
@@ -215,7 +224,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;Bs. OF&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -310,6 +319,19 @@
     <font>
       <u/>
       <sz val="12"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="14"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
@@ -550,7 +572,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="97">
+  <cellXfs count="104">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -740,6 +762,30 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -758,12 +804,6 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -782,18 +822,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -812,11 +840,26 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="4" fontId="17" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -839,238 +882,6 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>50800</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>257175</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>435429</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="Texto 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{55A93456-B5BC-4407-A826-D39FB9FF4A5E}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1">
-          <a:spLocks noChangeArrowheads="1"/>
-        </xdr:cNvSpPr>
-      </xdr:nvSpPr>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="3146425" y="2009775"/>
-          <a:ext cx="384629" cy="1295400"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="1">
-          <a:noFill/>
-          <a:miter lim="800000"/>
-          <a:headEnd/>
-          <a:tailEnd/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" vert="vert270" wrap="square" lIns="36576" tIns="32004" rIns="36576" bIns="32004" anchor="ctr" upright="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-VE" sz="1400" b="1" i="0" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Times New Roman"/>
-              <a:cs typeface="Times New Roman"/>
-            </a:rPr>
-            <a:t>CARGO</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>11906</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>241299</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>23813</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>36197</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="Texto 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C139C369-3F10-4647-9A32-154194F890E8}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1">
-          <a:spLocks noChangeArrowheads="1"/>
-        </xdr:cNvSpPr>
-      </xdr:nvSpPr>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="8555831" y="2003424"/>
-          <a:ext cx="773907" cy="1290323"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="1">
-          <a:noFill/>
-          <a:miter lim="800000"/>
-          <a:headEnd/>
-          <a:tailEnd/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" vert="vert270" wrap="square" lIns="36576" tIns="32004" rIns="36576" bIns="32004" anchor="ctr" upright="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-VE" sz="1200" b="1" i="0" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Times New Roman"/>
-              <a:cs typeface="Times New Roman"/>
-            </a:rPr>
-            <a:t>CATEG</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="es-VE" sz="1400" b="1" i="0" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Times New Roman"/>
-              <a:cs typeface="Times New Roman"/>
-            </a:rPr>
-            <a:t>.</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="ctr" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-VE" sz="1400" b="1" i="0" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Times New Roman"/>
-              <a:cs typeface="Times New Roman"/>
-            </a:rPr>
-            <a:t>DOCENTE</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>15875</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>473075</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="4" name="Texto 6">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{06181F22-F640-4954-A51F-0E0685BABBBC}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1">
-          <a:spLocks noChangeArrowheads="1"/>
-        </xdr:cNvSpPr>
-      </xdr:nvSpPr>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="6350000" y="2009775"/>
-          <a:ext cx="457200" cy="1295400"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="1">
-          <a:noFill/>
-          <a:miter lim="800000"/>
-          <a:headEnd/>
-          <a:tailEnd/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" vert="vert270" wrap="square" lIns="36576" tIns="27432" rIns="36576" bIns="27432" anchor="ctr" upright="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-VE" sz="1250" b="1" i="0" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Times New Roman"/>
-              <a:cs typeface="Times New Roman"/>
-            </a:rPr>
-            <a:t>Nº HORAS</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="ctr" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-VE" sz="1250" b="1" i="0" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Times New Roman"/>
-              <a:cs typeface="Times New Roman"/>
-            </a:rPr>
-            <a:t>SEMAN.</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>12</xdr:col>
@@ -1122,70 +933,6 @@
           </a:ext>
         </a:extLst>
       </xdr:spPr>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>90169</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>400985</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>79375</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="6" name="Texto 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CF591387-4A43-4041-A9C1-14E4A0B347A6}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1">
-          <a:spLocks noChangeArrowheads="1"/>
-        </xdr:cNvSpPr>
-      </xdr:nvSpPr>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="5919469" y="2019300"/>
-          <a:ext cx="310816" cy="1317625"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="1">
-          <a:noFill/>
-          <a:miter lim="800000"/>
-          <a:headEnd/>
-          <a:tailEnd/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" vert="vert270" wrap="square" lIns="36576" tIns="32004" rIns="36576" bIns="32004" anchor="ctr" upright="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr" rtl="0">
-            <a:defRPr sz="1000"/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="es-VE" sz="1400" b="1" i="0" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Times New Roman"/>
-              <a:cs typeface="Times New Roman"/>
-            </a:rPr>
-            <a:t>PUNTAJE</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
@@ -3004,15 +2751,15 @@
       <c r="M4" s="27"/>
       <c r="N4" s="24"/>
       <c r="O4" s="25"/>
-      <c r="P4" s="71"/>
-      <c r="Q4" s="71"/>
-      <c r="R4" s="71"/>
-      <c r="S4" s="71"/>
-      <c r="T4" s="71"/>
-      <c r="U4" s="71"/>
-      <c r="V4" s="71"/>
-      <c r="W4" s="71"/>
-      <c r="X4" s="72"/>
+      <c r="P4" s="79"/>
+      <c r="Q4" s="79"/>
+      <c r="R4" s="79"/>
+      <c r="S4" s="79"/>
+      <c r="T4" s="79"/>
+      <c r="U4" s="79"/>
+      <c r="V4" s="79"/>
+      <c r="W4" s="79"/>
+      <c r="X4" s="80"/>
       <c r="Y4" s="1"/>
       <c r="Z4" s="1"/>
       <c r="AA4" s="1"/>
@@ -3025,10 +2772,10 @@
       <c r="C5" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="73" t="s">
+      <c r="D5" s="81" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="74"/>
+      <c r="E5" s="82"/>
       <c r="F5" s="29" t="s">
         <v>8</v>
       </c>
@@ -3091,169 +2838,175 @@
       <c r="AA5" s="30"/>
     </row>
     <row r="6" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="75" t="s">
+      <c r="A6" s="83" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="75" t="s">
+      <c r="B6" s="83" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="77"/>
-      <c r="D6" s="79" t="s">
+      <c r="C6" s="99" t="s">
+        <v>56</v>
+      </c>
+      <c r="D6" s="85" t="s">
         <v>28</v>
       </c>
-      <c r="E6" s="80"/>
-      <c r="F6" s="83" t="s">
+      <c r="E6" s="86"/>
+      <c r="F6" s="89" t="s">
         <v>29</v>
       </c>
-      <c r="G6" s="77"/>
-      <c r="H6" s="77"/>
-      <c r="I6" s="85" t="s">
+      <c r="G6" s="97" t="s">
+        <v>55</v>
+      </c>
+      <c r="H6" s="97" t="s">
+        <v>57</v>
+      </c>
+      <c r="I6" s="75" t="s">
         <v>30</v>
       </c>
-      <c r="J6" s="85" t="s">
+      <c r="J6" s="102" t="s">
         <v>31</v>
       </c>
-      <c r="K6" s="77" t="s">
+      <c r="K6" s="97" t="s">
+        <v>58</v>
+      </c>
+      <c r="L6" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="L6" s="31" t="s">
+      <c r="M6" s="31"/>
+      <c r="N6" s="71" t="s">
         <v>33</v>
       </c>
-      <c r="M6" s="31"/>
-      <c r="N6" s="87" t="s">
+      <c r="O6" s="71" t="s">
         <v>34</v>
       </c>
-      <c r="O6" s="87" t="s">
+      <c r="P6" s="71" t="s">
         <v>35</v>
       </c>
-      <c r="P6" s="87" t="s">
+      <c r="Q6" s="71" t="s">
         <v>36</v>
       </c>
-      <c r="Q6" s="87" t="s">
+      <c r="R6" s="71" t="s">
         <v>37</v>
       </c>
-      <c r="R6" s="87" t="s">
+      <c r="S6" s="91" t="s">
         <v>38</v>
       </c>
-      <c r="S6" s="89" t="s">
+      <c r="T6" s="93" t="s">
         <v>39</v>
       </c>
-      <c r="T6" s="91" t="s">
+      <c r="U6" s="95" t="s">
         <v>40</v>
       </c>
-      <c r="U6" s="93" t="s">
+      <c r="V6" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="V6" s="32" t="s">
+      <c r="W6" s="77"/>
+      <c r="X6" s="93" t="s">
         <v>42</v>
-      </c>
-      <c r="W6" s="77"/>
-      <c r="X6" s="91" t="s">
-        <v>43</v>
       </c>
       <c r="Y6" s="33"/>
       <c r="Z6" s="33"/>
       <c r="AA6" s="33"/>
     </row>
     <row r="7" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="76"/>
-      <c r="B7" s="76"/>
-      <c r="C7" s="78"/>
-      <c r="D7" s="81"/>
-      <c r="E7" s="82"/>
-      <c r="F7" s="84"/>
-      <c r="G7" s="78"/>
-      <c r="H7" s="78"/>
-      <c r="I7" s="86"/>
-      <c r="J7" s="86"/>
-      <c r="K7" s="78"/>
+      <c r="A7" s="84"/>
+      <c r="B7" s="84"/>
+      <c r="C7" s="100"/>
+      <c r="D7" s="87"/>
+      <c r="E7" s="88"/>
+      <c r="F7" s="90"/>
+      <c r="G7" s="98"/>
+      <c r="H7" s="98"/>
+      <c r="I7" s="76"/>
+      <c r="J7" s="103"/>
+      <c r="K7" s="98"/>
       <c r="L7" s="34" t="s">
+        <v>43</v>
+      </c>
+      <c r="M7" s="34"/>
+      <c r="N7" s="72"/>
+      <c r="O7" s="72"/>
+      <c r="P7" s="72"/>
+      <c r="Q7" s="72"/>
+      <c r="R7" s="72"/>
+      <c r="S7" s="92"/>
+      <c r="T7" s="94"/>
+      <c r="U7" s="96"/>
+      <c r="V7" s="32" t="s">
         <v>44</v>
       </c>
-      <c r="M7" s="34"/>
-      <c r="N7" s="88"/>
-      <c r="O7" s="88"/>
-      <c r="P7" s="88"/>
-      <c r="Q7" s="88"/>
-      <c r="R7" s="88"/>
-      <c r="S7" s="90"/>
-      <c r="T7" s="92"/>
-      <c r="U7" s="94"/>
-      <c r="V7" s="32" t="s">
-        <v>45</v>
-      </c>
       <c r="W7" s="78"/>
-      <c r="X7" s="92"/>
+      <c r="X7" s="94"/>
       <c r="Y7" s="33"/>
       <c r="Z7" s="33"/>
       <c r="AA7" s="33"/>
     </row>
     <row r="8" spans="1:27" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="76"/>
-      <c r="B8" s="76"/>
-      <c r="C8" s="78"/>
-      <c r="D8" s="81"/>
-      <c r="E8" s="82"/>
-      <c r="F8" s="84"/>
-      <c r="G8" s="78"/>
-      <c r="H8" s="78"/>
-      <c r="I8" s="86"/>
-      <c r="J8" s="86"/>
-      <c r="K8" s="78"/>
+      <c r="A8" s="84"/>
+      <c r="B8" s="84"/>
+      <c r="C8" s="100"/>
+      <c r="D8" s="87"/>
+      <c r="E8" s="88"/>
+      <c r="F8" s="90"/>
+      <c r="G8" s="98"/>
+      <c r="H8" s="98"/>
+      <c r="I8" s="76"/>
+      <c r="J8" s="103"/>
+      <c r="K8" s="98"/>
       <c r="L8" s="35" t="s">
+        <v>45</v>
+      </c>
+      <c r="M8" s="35"/>
+      <c r="N8" s="72"/>
+      <c r="O8" s="72"/>
+      <c r="P8" s="72"/>
+      <c r="Q8" s="72"/>
+      <c r="R8" s="72"/>
+      <c r="S8" s="92"/>
+      <c r="T8" s="94"/>
+      <c r="U8" s="96"/>
+      <c r="V8" s="32" t="s">
         <v>46</v>
       </c>
-      <c r="M8" s="35"/>
-      <c r="N8" s="88"/>
-      <c r="O8" s="88"/>
-      <c r="P8" s="88"/>
-      <c r="Q8" s="88"/>
-      <c r="R8" s="88"/>
-      <c r="S8" s="90"/>
-      <c r="T8" s="92"/>
-      <c r="U8" s="94"/>
-      <c r="V8" s="32" t="s">
-        <v>47</v>
-      </c>
       <c r="W8" s="78"/>
-      <c r="X8" s="92"/>
+      <c r="X8" s="94"/>
       <c r="Y8" s="33"/>
       <c r="Z8" s="33"/>
       <c r="AA8" s="33"/>
     </row>
     <row r="9" spans="1:27" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="76"/>
-      <c r="B9" s="76"/>
-      <c r="C9" s="78"/>
+      <c r="A9" s="84"/>
+      <c r="B9" s="84"/>
+      <c r="C9" s="100"/>
       <c r="D9" s="36" t="s">
+        <v>47</v>
+      </c>
+      <c r="E9" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="E9" s="36" t="s">
+      <c r="F9" s="90"/>
+      <c r="G9" s="98"/>
+      <c r="H9" s="98"/>
+      <c r="I9" s="76"/>
+      <c r="J9" s="103"/>
+      <c r="K9" s="98"/>
+      <c r="L9" s="37" t="s">
         <v>49</v>
       </c>
-      <c r="F9" s="84"/>
-      <c r="G9" s="78"/>
-      <c r="H9" s="78"/>
-      <c r="I9" s="86"/>
-      <c r="J9" s="86"/>
-      <c r="K9" s="78"/>
-      <c r="L9" s="37" t="s">
+      <c r="M9" s="38" t="s">
         <v>50</v>
       </c>
-      <c r="M9" s="38" t="s">
-        <v>51</v>
-      </c>
-      <c r="N9" s="88"/>
-      <c r="O9" s="88"/>
-      <c r="P9" s="88"/>
-      <c r="Q9" s="88"/>
-      <c r="R9" s="88"/>
-      <c r="S9" s="90"/>
-      <c r="T9" s="92"/>
-      <c r="U9" s="94"/>
+      <c r="N9" s="72"/>
+      <c r="O9" s="72"/>
+      <c r="P9" s="72"/>
+      <c r="Q9" s="72"/>
+      <c r="R9" s="72"/>
+      <c r="S9" s="92"/>
+      <c r="T9" s="94"/>
+      <c r="U9" s="96"/>
       <c r="V9" s="32"/>
       <c r="W9" s="78"/>
-      <c r="X9" s="92"/>
+      <c r="X9" s="94"/>
       <c r="Y9" s="33"/>
       <c r="Z9" s="33"/>
       <c r="AA9" s="33"/>
@@ -3419,7 +3172,7 @@
       <c r="M15" s="39"/>
       <c r="N15" s="40"/>
       <c r="O15" s="40"/>
-      <c r="P15" s="40"/>
+      <c r="P15" s="101"/>
       <c r="Q15" s="41"/>
       <c r="R15" s="41"/>
       <c r="S15" s="41"/>
@@ -5039,10 +4792,10 @@
       <c r="I71" s="33"/>
       <c r="J71" s="33"/>
       <c r="K71" s="33"/>
-      <c r="M71" s="95" t="s">
-        <v>52</v>
-      </c>
-      <c r="N71" s="96"/>
+      <c r="M71" s="73" t="s">
+        <v>51</v>
+      </c>
+      <c r="N71" s="74"/>
       <c r="O71" s="53">
         <f>SUM(O10:O69)</f>
         <v>0</v>
@@ -5145,7 +4898,7 @@
     </row>
     <row r="74" spans="1:27" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A74" s="54" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B74" s="55"/>
       <c r="C74" s="56"/>
@@ -5205,7 +4958,7 @@
     </row>
     <row r="76" spans="1:27" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A76" s="61" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B76" s="55"/>
       <c r="C76" s="56"/>
@@ -5255,7 +5008,7 @@
       <c r="V77" s="17"/>
       <c r="W77" s="17"/>
       <c r="X77" s="58" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="Y77" s="33"/>
       <c r="Z77" s="33"/>
@@ -5295,13 +5048,6 @@
     </row>
   </sheetData>
   <mergeCells count="23">
-    <mergeCell ref="Q6:Q9"/>
-    <mergeCell ref="M71:N71"/>
-    <mergeCell ref="J6:J9"/>
-    <mergeCell ref="K6:K9"/>
-    <mergeCell ref="N6:N9"/>
-    <mergeCell ref="O6:O9"/>
-    <mergeCell ref="P6:P9"/>
     <mergeCell ref="P4:X4"/>
     <mergeCell ref="D5:E5"/>
     <mergeCell ref="A6:A9"/>
@@ -5318,6 +5064,13 @@
     <mergeCell ref="U6:U9"/>
     <mergeCell ref="W6:W9"/>
     <mergeCell ref="X6:X9"/>
+    <mergeCell ref="Q6:Q9"/>
+    <mergeCell ref="M71:N71"/>
+    <mergeCell ref="J6:J9"/>
+    <mergeCell ref="K6:K9"/>
+    <mergeCell ref="N6:N9"/>
+    <mergeCell ref="O6:O9"/>
+    <mergeCell ref="P6:P9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="38" orientation="landscape" r:id="rId1"/>

</xml_diff>